<commit_message>
Prioritize fewer pieces/plates over waste in nesting and pricing
Switch the default objective to "convenience" (fewest pieces per panel,
then fewest plates, then cost), add a cost-optimal comparison, and report
plates-to-buy per type. Aligns equal panels to the same plate/price.

https://claude.ai/code/session_01KNfHFGm3BZAV2u3TfGKXLF
</commit_message>
<xml_diff>
--- a/pricing.xlsx
+++ b/pricing.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="תמחור" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="לוחות לקנייה" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -499,23 +500,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>הצעת מחיר - פאנלים (כולל 30% רווח)</t>
+          <t>הצעת מחיר - עדיפות נוחות עבודה (כולל 30% רווח)</t>
         </is>
       </c>
     </row>
@@ -537,25 +539,30 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>חתיכות לפאנל</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>לוחות</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>עלות חומר</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>עלות ליחידה</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>מחיר מכירה ליחידה</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>סה״כ מכירה</t>
         </is>
@@ -572,23 +579,26 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>1250x2500</t>
+          <t>1500x3000</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>2760</v>
+        <v>3</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>12</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>460</v>
-      </c>
-      <c r="G3" s="5" t="n">
-        <v>598</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>3588</v>
+        <v>3720</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>620</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>806</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>4836</v>
       </c>
     </row>
     <row r="4">
@@ -602,23 +612,26 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>1000x3000</t>
+          <t>1500x3000</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>1472</v>
+        <v>3</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>6</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>490.7</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>638</v>
-      </c>
-      <c r="H4" s="6" t="n">
-        <v>1914</v>
+        <v>1860</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>620</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>806</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>2418</v>
       </c>
     </row>
     <row r="5">
@@ -636,18 +649,21 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>552</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="G5" s="4" t="n">
         <v>92</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="H5" s="5" t="n">
         <v>120</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="I5" s="6" t="n">
         <v>720</v>
       </c>
     </row>
@@ -666,18 +682,21 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>1656</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="G6" s="4" t="n">
         <v>552</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="H6" s="5" t="n">
         <v>718</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="I6" s="6" t="n">
         <v>2154</v>
       </c>
     </row>
@@ -696,18 +715,21 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>3312</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="G7" s="4" t="n">
         <v>552</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="H7" s="5" t="n">
         <v>718</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="I7" s="6" t="n">
         <v>4308</v>
       </c>
     </row>
@@ -722,23 +744,26 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>1000x2000</t>
+          <t>1000x3000</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>366</v>
+        <v>1</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>61</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>79</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>474</v>
+        <v>368</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>480</v>
       </c>
     </row>
     <row r="9">
@@ -752,23 +777,26 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>1000x2000</t>
+          <t>1000x3000</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>2196</v>
+        <v>2</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>12</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>366</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>476</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>2856</v>
+        <v>2208</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>368</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>478</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>2868</v>
       </c>
     </row>
     <row r="10">
@@ -786,18 +814,21 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>3720</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="G10" s="4" t="n">
         <v>310</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="H10" s="5" t="n">
         <v>403</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="I10" s="6" t="n">
         <v>4836</v>
       </c>
     </row>
@@ -812,23 +843,26 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>1000x2000</t>
+          <t>1500x3000</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>488</v>
+        <v>1</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>40.7</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>53</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>636</v>
+        <v>620</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>804</v>
       </c>
     </row>
     <row r="12">
@@ -837,63 +871,161 @@
           <t>סה״כ</t>
         </is>
       </c>
-      <c r="E12" s="8" t="n">
-        <v>16522</v>
-      </c>
-      <c r="F12" s="9" t="n"/>
+      <c r="F12" s="8" t="n">
+        <v>18016</v>
+      </c>
       <c r="G12" s="9" t="n"/>
-      <c r="H12" s="10" t="n">
-        <v>21486</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>עלות חומר (תמחור עצמאי):</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>16522</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>עלות חומר בפועל (אריזה משותפת):</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="n">
-        <v>15910</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="10" t="n">
+        <v>23424</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A12:E12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>לוחות לקנייה (תכנון נוחות)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>פלטה (מ״מ)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>כמות לוחות</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>עלות (₪)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>1000x3000</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>7544</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>1250x2500</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>1500x3000</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>9610</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>סה״כ</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>17706</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>עלות חומר - תכנון נוחות:</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>17706</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>עלות חומר - תכנון זול-ביותר:</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>16278</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>תוספת עבור נוחות:</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>1428</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>סה״כ הצעת מחיר (כולל 30%):</t>
         </is>
       </c>
-      <c r="E16" s="10" t="n">
-        <v>21486</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>רווח גולמי מעל עלות בפועל:</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="n">
-        <v>5576</v>
+      <c r="C11" s="10" t="n">
+        <v>23424</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A14:D14"/>
+  <mergeCells count="5">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A8:B8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>